<commit_message>
commit final for the week added comparison button
</commit_message>
<xml_diff>
--- a/BSE/FnO/bse_fno_consolidated.xlsx
+++ b/BSE/FnO/bse_fno_consolidated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1506"/>
+  <dimension ref="A1:O1508"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -78118,6 +78118,160 @@
         </is>
       </c>
     </row>
+    <row r="1507">
+      <c r="A1507" t="inlineStr">
+        <is>
+          <t>18-Feb-2026</t>
+        </is>
+      </c>
+      <c r="B1507" t="inlineStr">
+        <is>
+          <t>3,28,26,032</t>
+        </is>
+      </c>
+      <c r="C1507" t="inlineStr">
+        <is>
+          <t>12,12,87,581</t>
+        </is>
+      </c>
+      <c r="D1507" t="inlineStr">
+        <is>
+          <t>2,02,56,507.92</t>
+        </is>
+      </c>
+      <c r="E1507" t="inlineStr">
+        <is>
+          <t>31,391.93</t>
+        </is>
+      </c>
+      <c r="F1507" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G1507" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1507" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="I1507" t="inlineStr">
+        <is>
+          <t>1,107</t>
+        </is>
+      </c>
+      <c r="J1507" t="inlineStr">
+        <is>
+          <t>1,377</t>
+        </is>
+      </c>
+      <c r="K1507" t="inlineStr">
+        <is>
+          <t>230.41</t>
+        </is>
+      </c>
+      <c r="L1507" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="M1507" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="N1507" t="inlineStr">
+        <is>
+          <t>0.45</t>
+        </is>
+      </c>
+      <c r="O1507" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+    </row>
+    <row r="1508">
+      <c r="A1508" t="inlineStr">
+        <is>
+          <t>19-Feb-2026</t>
+        </is>
+      </c>
+      <c r="B1508" t="inlineStr">
+        <is>
+          <t>9,99,82,199</t>
+        </is>
+      </c>
+      <c r="C1508" t="inlineStr">
+        <is>
+          <t>52,22,88,476</t>
+        </is>
+      </c>
+      <c r="D1508" t="inlineStr">
+        <is>
+          <t>8,68,52,466.01</t>
+        </is>
+      </c>
+      <c r="E1508" t="inlineStr">
+        <is>
+          <t>59,310.34</t>
+        </is>
+      </c>
+      <c r="F1508" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G1508" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1508" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="I1508" t="inlineStr">
+        <is>
+          <t>2,316</t>
+        </is>
+      </c>
+      <c r="J1508" t="inlineStr">
+        <is>
+          <t>2,827</t>
+        </is>
+      </c>
+      <c r="K1508" t="inlineStr">
+        <is>
+          <t>470.07</t>
+        </is>
+      </c>
+      <c r="L1508" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="M1508" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="N1508" t="inlineStr">
+        <is>
+          <t>0.26</t>
+        </is>
+      </c>
+      <c r="O1508" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>